<commit_message>
Nuevo dominio con digitalplat y URL en imagen del logo del cliente
</commit_message>
<xml_diff>
--- a/plantilla_sitio.xlsx
+++ b/plantilla_sitio.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CW41"/>
+  <dimension ref="A1:CW43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -498,7 +498,7 @@
     <col width="22" customWidth="1" min="29" max="29"/>
     <col width="24" customWidth="1" min="30" max="30"/>
     <col width="27" customWidth="1" min="31" max="31"/>
-    <col width="30" customWidth="1" min="32" max="32"/>
+    <col width="50" customWidth="1" min="32" max="32"/>
     <col width="25" customWidth="1" min="33" max="33"/>
     <col width="18" customWidth="1" min="34" max="34"/>
     <col width="18" customWidth="1" min="35" max="35"/>
@@ -7907,6 +7907,284 @@
       <c r="CV41" s="2" t="n"/>
       <c r="CW41" s="2" t="n"/>
     </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>802-SV-001</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>INSTRUMENTOS</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Válvula solenoide</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Ingreso/cierre de  aire de la bomba neumatica 802-P-01 (Floculante)</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Continua</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Aire comprimido</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="n"/>
+      <c r="I42" s="2" t="n"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>&lt;30</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="n"/>
+      <c r="L42" s="2" t="n"/>
+      <c r="M42" s="2" t="n"/>
+      <c r="N42" s="2" t="n"/>
+      <c r="O42" s="2" t="n"/>
+      <c r="P42" s="2" t="n"/>
+      <c r="Q42" s="2" t="n"/>
+      <c r="R42" s="2" t="n"/>
+      <c r="S42" s="2" t="n"/>
+      <c r="T42" s="2" t="n"/>
+      <c r="U42" s="2" t="n"/>
+      <c r="V42" s="2" t="n"/>
+      <c r="W42" s="2" t="n"/>
+      <c r="X42" s="2" t="n"/>
+      <c r="Y42" s="2" t="n"/>
+      <c r="Z42" s="2" t="n"/>
+      <c r="AA42" s="2" t="n"/>
+      <c r="AB42" s="2" t="n"/>
+      <c r="AC42" s="2" t="n"/>
+      <c r="AD42" s="2" t="n"/>
+      <c r="AE42" s="2" t="n"/>
+      <c r="AF42" s="2" t="inlineStr">
+        <is>
+          <t>Válvula solenoide con actuador neumático. Presión de suministro de aire: 29 ---145</t>
+        </is>
+      </c>
+      <c r="AG42" s="2" t="n"/>
+      <c r="AH42" s="2" t="n"/>
+      <c r="AI42" s="2" t="n"/>
+      <c r="AJ42" s="2" t="n"/>
+      <c r="AK42" s="2" t="n"/>
+      <c r="AL42" s="2" t="n"/>
+      <c r="AM42" s="2" t="n"/>
+      <c r="AN42" s="2" t="n"/>
+      <c r="AO42" s="2" t="n"/>
+      <c r="AP42" s="2" t="n"/>
+      <c r="AQ42" s="2" t="n"/>
+      <c r="AR42" s="2" t="n"/>
+      <c r="AS42" s="2" t="n"/>
+      <c r="AT42" s="2" t="n"/>
+      <c r="AU42" s="2" t="n"/>
+      <c r="AV42" s="2" t="n"/>
+      <c r="AW42" s="2" t="n"/>
+      <c r="AX42" s="2" t="n"/>
+      <c r="AY42" s="2" t="n"/>
+      <c r="AZ42" s="2" t="n"/>
+      <c r="BA42" s="2" t="n"/>
+      <c r="BB42" s="2" t="n"/>
+      <c r="BC42" s="2" t="n"/>
+      <c r="BD42" s="2" t="n"/>
+      <c r="BE42" s="2" t="n"/>
+      <c r="BF42" s="2" t="n"/>
+      <c r="BG42" s="2" t="n"/>
+      <c r="BH42" s="2" t="n"/>
+      <c r="BI42" s="2" t="n"/>
+      <c r="BJ42" s="2" t="n"/>
+      <c r="BK42" s="2" t="n"/>
+      <c r="BL42" s="2" t="n"/>
+      <c r="BM42" s="2" t="n"/>
+      <c r="BN42" s="2" t="n"/>
+      <c r="BO42" s="2" t="n"/>
+      <c r="BP42" s="2" t="n"/>
+      <c r="BQ42" s="2" t="n"/>
+      <c r="BR42" s="2" t="n"/>
+      <c r="BS42" s="2" t="n"/>
+      <c r="BT42" s="2" t="n"/>
+      <c r="BU42" s="2" t="n"/>
+      <c r="BV42" s="2" t="n"/>
+      <c r="BW42" s="2" t="n"/>
+      <c r="BX42" s="2" t="n"/>
+      <c r="BY42" s="2" t="n"/>
+      <c r="BZ42" s="2" t="n"/>
+      <c r="CA42" s="2" t="n"/>
+      <c r="CB42" s="2" t="n"/>
+      <c r="CC42" s="2" t="n"/>
+      <c r="CD42" s="2" t="n"/>
+      <c r="CE42" s="2" t="n"/>
+      <c r="CF42" s="2" t="n"/>
+      <c r="CG42" s="2" t="n"/>
+      <c r="CH42" s="2" t="n"/>
+      <c r="CI42" s="2" t="n"/>
+      <c r="CJ42" s="2" t="n"/>
+      <c r="CK42" s="2" t="n"/>
+      <c r="CL42" s="2" t="n"/>
+      <c r="CM42" s="2" t="n"/>
+      <c r="CN42" s="2" t="n"/>
+      <c r="CO42" s="2" t="n"/>
+      <c r="CP42" s="2" t="n"/>
+      <c r="CQ42" s="2" t="n"/>
+      <c r="CR42" s="2" t="n"/>
+      <c r="CS42" s="2" t="n"/>
+      <c r="CT42" s="2" t="n"/>
+      <c r="CU42" s="2" t="inlineStr">
+        <is>
+          <t>20 - 25</t>
+        </is>
+      </c>
+      <c r="CV42" s="2" t="n"/>
+      <c r="CW42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>600-SV-01</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>INSTRUMENTOS</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Válvula solenoide</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Ingreso/cierre de  aire Línea de aire comprimido hacia bomba 600-P-01 (Trasiego de lodos)</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Discontinua</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Aire comprimido</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="n"/>
+      <c r="I43" s="2" t="n"/>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>&lt;30</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="n"/>
+      <c r="L43" s="2" t="n"/>
+      <c r="M43" s="2" t="n"/>
+      <c r="N43" s="2" t="n"/>
+      <c r="O43" s="2" t="n"/>
+      <c r="P43" s="2" t="n"/>
+      <c r="Q43" s="2" t="n"/>
+      <c r="R43" s="2" t="n"/>
+      <c r="S43" s="2" t="n"/>
+      <c r="T43" s="2" t="n"/>
+      <c r="U43" s="2" t="n"/>
+      <c r="V43" s="2" t="n"/>
+      <c r="W43" s="2" t="n"/>
+      <c r="X43" s="2" t="n"/>
+      <c r="Y43" s="2" t="n"/>
+      <c r="Z43" s="2" t="n"/>
+      <c r="AA43" s="2" t="n"/>
+      <c r="AB43" s="2" t="n"/>
+      <c r="AC43" s="2" t="n"/>
+      <c r="AD43" s="2" t="n"/>
+      <c r="AE43" s="2" t="n"/>
+      <c r="AF43" s="2" t="inlineStr">
+        <is>
+          <t>Válvula solenoide con actuador eléctrico</t>
+        </is>
+      </c>
+      <c r="AG43" s="2" t="n"/>
+      <c r="AH43" s="2" t="n"/>
+      <c r="AI43" s="2" t="n"/>
+      <c r="AJ43" s="2" t="n"/>
+      <c r="AK43" s="2" t="n"/>
+      <c r="AL43" s="2" t="n"/>
+      <c r="AM43" s="2" t="n"/>
+      <c r="AN43" s="2" t="n"/>
+      <c r="AO43" s="2" t="n"/>
+      <c r="AP43" s="2" t="n"/>
+      <c r="AQ43" s="2" t="n"/>
+      <c r="AR43" s="2" t="n"/>
+      <c r="AS43" s="2" t="n"/>
+      <c r="AT43" s="2" t="n"/>
+      <c r="AU43" s="2" t="n"/>
+      <c r="AV43" s="2" t="n"/>
+      <c r="AW43" s="2" t="n"/>
+      <c r="AX43" s="2" t="n"/>
+      <c r="AY43" s="2" t="n"/>
+      <c r="AZ43" s="2" t="n"/>
+      <c r="BA43" s="2" t="n"/>
+      <c r="BB43" s="2" t="n"/>
+      <c r="BC43" s="2" t="n"/>
+      <c r="BD43" s="2" t="n"/>
+      <c r="BE43" s="2" t="n"/>
+      <c r="BF43" s="2" t="n"/>
+      <c r="BG43" s="2" t="n"/>
+      <c r="BH43" s="2" t="n"/>
+      <c r="BI43" s="2" t="n"/>
+      <c r="BJ43" s="2" t="n"/>
+      <c r="BK43" s="2" t="n"/>
+      <c r="BL43" s="2" t="n"/>
+      <c r="BM43" s="2" t="n"/>
+      <c r="BN43" s="2" t="n"/>
+      <c r="BO43" s="2" t="n"/>
+      <c r="BP43" s="2" t="n"/>
+      <c r="BQ43" s="2" t="n"/>
+      <c r="BR43" s="2" t="n"/>
+      <c r="BS43" s="2" t="n"/>
+      <c r="BT43" s="2" t="n"/>
+      <c r="BU43" s="2" t="n"/>
+      <c r="BV43" s="2" t="n"/>
+      <c r="BW43" s="2" t="n"/>
+      <c r="BX43" s="2" t="n"/>
+      <c r="BY43" s="2" t="n"/>
+      <c r="BZ43" s="2" t="n"/>
+      <c r="CA43" s="2" t="n"/>
+      <c r="CB43" s="2" t="n"/>
+      <c r="CC43" s="2" t="n"/>
+      <c r="CD43" s="2" t="n"/>
+      <c r="CE43" s="2" t="n"/>
+      <c r="CF43" s="2" t="n"/>
+      <c r="CG43" s="2" t="n"/>
+      <c r="CH43" s="2" t="n"/>
+      <c r="CI43" s="2" t="n"/>
+      <c r="CJ43" s="2" t="n"/>
+      <c r="CK43" s="2" t="n"/>
+      <c r="CL43" s="2" t="n"/>
+      <c r="CM43" s="2" t="n"/>
+      <c r="CN43" s="2" t="n"/>
+      <c r="CO43" s="2" t="n"/>
+      <c r="CP43" s="2" t="n"/>
+      <c r="CQ43" s="2" t="n"/>
+      <c r="CR43" s="2" t="n"/>
+      <c r="CS43" s="2" t="n"/>
+      <c r="CT43" s="2" t="n"/>
+      <c r="CU43" s="2" t="inlineStr">
+        <is>
+          <t>20 - 25</t>
+        </is>
+      </c>
+      <c r="CV43" s="2" t="n"/>
+      <c r="CW43" s="2" t="n"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Categoría inválida" error="Debe ser una de: EQUIPOS, INSTRUMENTOS, TANQUES" promptTitle="Categoría" prompt="Selecciona: EQUIPOS, INSTRUMENTOS, TANQUES" type="list">

</xml_diff>